<commit_message>
T2: show-your-work brought to the house register
Counts in words, 2,080 with its comma, no parentheticals, family labels as the metadata names
them, dollars formatted as the documents write them; the read-back guard and its control follow.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BFcAyctgtHUfeGuTMXxq24
</commit_message>
<xml_diff>
--- a/tasks/HR_Troutly_T2_pto_liability_close/03_show_your_work.xlsx
+++ b/tasks/HR_Troutly_T2_pto_liability_close/03_show_your_work.xlsx
@@ -449,7 +449,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Biweekly accrual at the annual tier over 26, posted on the pay date; carryover capped at 40.0 hours at 06/30/2026; tiers by adjusted service date, the change in the period containing the anniversary; valued at the rate on file over 2080; ended employees out; wiki pages do not set policy.</t>
+          <t>Biweekly accrual at the annual tier over 26, posted on the pay date; carryover capped at 40.0 hours at 06/30/2026; tiers by adjusted service date, the change in the period containing the anniversary; valued at the rate on file over 2,080; ended employees out; wiki pages do not set policy.</t>
         </is>
       </c>
     </row>
@@ -500,7 +500,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>52 active employees. BambooHR carries 57 active rows: four contractors, three ended employees (03/20, 05/08 and 06/15/2026) and no row for TRT-0153 and TRT-0155, Never Loaded on the crosswalk.</t>
+          <t>52 active employees. BambooHR carries 57 active rows: four contractors, three employees whose employment ended 03/20, 05/08 and 06/15/2026, and no row for TRT-0153 and TRT-0155, Never Loaded on the crosswalk.</t>
         </is>
       </c>
     </row>
@@ -517,7 +517,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>51 balances at 06/30/2026; 11 above 40.0 hours, TRT-0005 at 92.50 the highest. The HRIS report, the load file and the July close carry them uncapped.</t>
+          <t>51 balances at 06/30/2026; eleven above 40.0 hours, TRT-0005 at 92.50 the highest. The HRIS report, the load file and the July close carry them uncapped.</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Pay dates 07/10/2026, 07/24/2026, 08/07/2026, 08/21/2026 by 08/31/2026; 09/04/2026 is the fifth and is not posted.</t>
+          <t>Pay dates 07/10/2026, 07/24/2026, 08/07/2026 and 08/21/2026, posted by 08/31/2026; 09/04/2026 is the fifth and is not posted.</t>
         </is>
       </c>
     </row>
@@ -551,7 +551,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>9 migrated records read 07/01/2026 in BambooHR and on the roster and carry their true dates in the archive and the letters. TRT-0071 hired 03/08/2021, ended 08/25/2023, rehired 04/22/2024: a break under 365 days, bridged under handbook 7.6.</t>
+          <t>Nine migrated records read 07/01/2026 in BambooHR and on the roster and carry their true dates in the archive and the letters. TRT-0071 hired 03/08/2021, ended 08/25/2023, rehired 04/22/2024: a break under 365 days, bridged under handbook 7.6.</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Historical offer letters, Marchetti, and handbook 5.4</t>
+          <t>Marchetti's offer letter in the historical letters and handbook 5.4</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -631,7 +631,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>The roster, the signed offers, /Recruiting/Offers/2026-07-02_Offer_TRT-0153_SIGNED.pdf and letter 13 of the historical letters, and Greenhouse</t>
+          <t>The roster, the signed offer /Recruiting/Offers/2026-07-02_Offer_TRT-0153_SIGNED.pdf, letter 13 of the historical letters and Greenhouse</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -687,7 +687,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>57 active rows, the loaded policies (6 wrong) and the loaded balances the run brings to the schedule.</t>
+          <t>57 active rows, the loaded policies, six of them wrong, and the loaded balances the run brings to the schedule.</t>
         </is>
       </c>
     </row>
@@ -743,7 +743,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>free</t>
+          <t>The page and its form</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -766,7 +766,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>free</t>
+          <t>The page and its form</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -789,7 +789,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>free</t>
+          <t>The page and its form</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -812,7 +812,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>free</t>
+          <t>The page and its form</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -835,7 +835,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>determination</t>
+          <t>The determination</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -858,7 +858,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>determination</t>
+          <t>The determination</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -881,7 +881,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>determination</t>
+          <t>The determination</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -904,7 +904,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>determination</t>
+          <t>The determination</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -927,7 +927,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>determination</t>
+          <t>The determination</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -950,7 +950,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>determination</t>
+          <t>The determination</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -973,7 +973,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>determination</t>
+          <t>The determination</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -996,7 +996,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>determination</t>
+          <t>The determination</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -1019,7 +1019,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>determination</t>
+          <t>The determination</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1042,7 +1042,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>determination</t>
+          <t>The determination</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1065,7 +1065,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>determination</t>
+          <t>The determination</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -1088,7 +1088,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>determination</t>
+          <t>The determination</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -1111,7 +1111,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>determination</t>
+          <t>The determination</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1134,7 +1134,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>determination</t>
+          <t>The determination</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1157,7 +1157,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>bamboohr</t>
+          <t>BambooHR brought to the schedule</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -1180,7 +1180,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>bamboohr</t>
+          <t>BambooHR brought to the schedule</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -1203,7 +1203,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>bamboohr</t>
+          <t>BambooHR brought to the schedule</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -1286,7 +1286,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>The archive's 06/30/2026 balance capped at 40.00; 11 capped; the two hires at 0.00.</t>
+          <t>The archive's 06/30/2026 balance capped at 40.00; eleven capped; the two hires at 0.00.</t>
         </is>
       </c>
     </row>
@@ -1334,7 +1334,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>The rate on file over 2080 to four decimals: TRT-0088 at $118,000.00, TRT-0117 at $148,200.00 and TRT-0096 at $61,000.00 by the signed documents and the step.</t>
+          <t>The rate on file over 2,080 to four decimals: TRT-0088 at $118,000.00, TRT-0117 at $148,200.00 and TRT-0096 at $61,000.00 by the signed documents and the step.</t>
         </is>
       </c>
     </row>
@@ -1346,7 +1346,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Balance to two decimals, liability to the cent, the total the sum of the rounded rows: 1,522.17 hours and $92,739.54 ($92,772.88 under posted rounding).</t>
+          <t>Balance to two decimals, liability to the cent, the total the sum of the rounded rows: 1,522.17 hours and $92,739.54, $92,772.88 under posted rounding.</t>
         </is>
       </c>
     </row>
@@ -1370,7 +1370,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>6 policies reassigned, 52 balances set, rows created for TRT-0153 and TRT-0155.</t>
+          <t>Six policies reassigned, 52 balances set, rows created for TRT-0153 and TRT-0155.</t>
         </is>
       </c>
     </row>
@@ -1546,17 +1546,17 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>215000.00</t>
+          <t>$215,000.00</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>103.3654</t>
+          <t>$103.3654</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2363.97</t>
+          <t>$2,363.97</t>
         </is>
       </c>
     </row>
@@ -1631,17 +1631,17 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>205000.00</t>
+          <t>$205,000.00</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>98.5577</t>
+          <t>$98.5577</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>6171.68</t>
+          <t>$6,171.68</t>
         </is>
       </c>
     </row>
@@ -1716,17 +1716,17 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>187510.00</t>
+          <t>$187,510.00</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>90.1490</t>
+          <t>$90.1490</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>5825.43</t>
+          <t>$5,825.43</t>
         </is>
       </c>
     </row>
@@ -1801,17 +1801,17 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>138700.00</t>
+          <t>$138,700.00</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>66.6827</t>
+          <t>$66.6827</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>4309.04</t>
+          <t>$4,309.04</t>
         </is>
       </c>
     </row>
@@ -1886,17 +1886,17 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>176400.00</t>
+          <t>$176,400.00</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>84.8077</t>
+          <t>$84.8077</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>1565.55</t>
+          <t>$1,565.55</t>
         </is>
       </c>
     </row>
@@ -1971,17 +1971,17 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>156700.00</t>
+          <t>$156,700.00</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>75.3365</t>
+          <t>$75.3365</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>4404.17</t>
+          <t>$4,404.17</t>
         </is>
       </c>
     </row>
@@ -2056,17 +2056,17 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>173300.00</t>
+          <t>$173,300.00</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>83.3173</t>
+          <t>$83.3173</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>4999.04</t>
+          <t>$4,999.04</t>
         </is>
       </c>
     </row>
@@ -2141,17 +2141,17 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>121300.00</t>
+          <t>$121,300.00</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>58.3173</t>
+          <t>$58.3173</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>2476.15</t>
+          <t>$2,476.15</t>
         </is>
       </c>
     </row>
@@ -2226,17 +2226,17 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>154900.00</t>
+          <t>$154,900.00</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>74.4712</t>
+          <t>$74.4712</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>4353.59</t>
+          <t>$4,353.59</t>
         </is>
       </c>
     </row>
@@ -2311,17 +2311,17 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>157600.00</t>
+          <t>$157,600.00</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>75.7692</t>
+          <t>$75.7692</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>2023.80</t>
+          <t>$2,023.80</t>
         </is>
       </c>
     </row>
@@ -2396,17 +2396,17 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>101400.00</t>
+          <t>$101,400.00</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>48.7500</t>
+          <t>$48.7500</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>2459.93</t>
+          <t>$2,459.93</t>
         </is>
       </c>
     </row>
@@ -2481,17 +2481,17 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>161200.00</t>
+          <t>$161,200.00</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>77.5000</t>
+          <t>$77.5000</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>2050.65</t>
+          <t>$2,050.65</t>
         </is>
       </c>
     </row>
@@ -2566,17 +2566,17 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>84600.00</t>
+          <t>$84,600.00</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>40.6731</t>
+          <t>$40.6731</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>1259.24</t>
+          <t>$1,259.24</t>
         </is>
       </c>
     </row>
@@ -2651,17 +2651,17 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>176400.00</t>
+          <t>$176,400.00</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>84.8077</t>
+          <t>$84.8077</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>4957.86</t>
+          <t>$4,957.86</t>
         </is>
       </c>
     </row>
@@ -2736,17 +2736,17 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>97350.00</t>
+          <t>$97,350.00</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>46.8029</t>
+          <t>$46.8029</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>1612.83</t>
+          <t>$1,612.83</t>
         </is>
       </c>
     </row>
@@ -2821,17 +2821,17 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>100800.00</t>
+          <t>$100,800.00</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>48.4615</t>
+          <t>$48.4615</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>385.75</t>
+          <t>$385.75</t>
         </is>
       </c>
     </row>
@@ -2906,17 +2906,17 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>132300.00</t>
+          <t>$132,300.00</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>63.6058</t>
+          <t>$63.6058</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>347.29</t>
+          <t>$347.29</t>
         </is>
       </c>
     </row>
@@ -2991,17 +2991,17 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>129800.00</t>
+          <t>$129,800.00</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>62.4038</t>
+          <t>$62.4038</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>418.73</t>
+          <t>$418.73</t>
         </is>
       </c>
     </row>
@@ -3076,17 +3076,17 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>103700.00</t>
+          <t>$103,700.00</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>49.8558</t>
+          <t>$49.8558</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>222.36</t>
+          <t>$222.36</t>
         </is>
       </c>
     </row>
@@ -3161,17 +3161,17 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>130450.00</t>
+          <t>$130,450.00</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>62.7163</t>
+          <t>$62.7163</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>1000.95</t>
+          <t>$1,000.95</t>
         </is>
       </c>
     </row>
@@ -3246,17 +3246,17 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>94750.00</t>
+          <t>$94,750.00</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>45.5529</t>
+          <t>$45.5529</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>1865.85</t>
+          <t>$1,865.85</t>
         </is>
       </c>
     </row>
@@ -3331,17 +3331,17 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>152600.00</t>
+          <t>$152,600.00</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>73.3654</t>
+          <t>$73.3654</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>1556.08</t>
+          <t>$1,556.08</t>
         </is>
       </c>
     </row>
@@ -3416,17 +3416,17 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>179800.00</t>
+          <t>$179,800.00</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>86.4423</t>
+          <t>$86.4423</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>2416.93</t>
+          <t>$2,416.93</t>
         </is>
       </c>
     </row>
@@ -3501,17 +3501,17 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>99300.00</t>
+          <t>$99,300.00</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>47.7404</t>
+          <t>$47.7404</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>2206.08</t>
+          <t>$2,206.08</t>
         </is>
       </c>
     </row>
@@ -3586,17 +3586,17 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>81000.00</t>
+          <t>$81,000.00</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t>38.9423</t>
+          <t>$38.9423</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>2019.94</t>
+          <t>$2,019.94</t>
         </is>
       </c>
     </row>
@@ -3671,17 +3671,17 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>111800.00</t>
+          <t>$111,800.00</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t>53.7500</t>
+          <t>$53.7500</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>2376.29</t>
+          <t>$2,376.29</t>
         </is>
       </c>
     </row>
@@ -3756,17 +3756,17 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>151900.00</t>
+          <t>$151,900.00</t>
         </is>
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>73.0288</t>
+          <t>$73.0288</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>2571.34</t>
+          <t>$2,571.34</t>
         </is>
       </c>
     </row>
@@ -3841,17 +3841,17 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>119600.00</t>
+          <t>$119,600.00</t>
         </is>
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>57.5000</t>
+          <t>$57.5000</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>1435.20</t>
+          <t>$1,435.20</t>
         </is>
       </c>
     </row>
@@ -3926,17 +3926,17 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>93100.00</t>
+          <t>$93,100.00</t>
         </is>
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>44.7596</t>
+          <t>$44.7596</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>837.45</t>
+          <t>$837.45</t>
         </is>
       </c>
     </row>
@@ -4011,17 +4011,17 @@
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>63750.00</t>
+          <t>$63,750.00</t>
         </is>
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>30.6490</t>
+          <t>$30.6490</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>1592.52</t>
+          <t>$1,592.52</t>
         </is>
       </c>
     </row>
@@ -4096,17 +4096,17 @@
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>118000.00</t>
+          <t>$118,000.00</t>
         </is>
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>56.7308</t>
+          <t>$56.7308</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>749.41</t>
+          <t>$749.41</t>
         </is>
       </c>
     </row>
@@ -4181,17 +4181,17 @@
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>144500.00</t>
+          <t>$144,500.00</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>69.4712</t>
+          <t>$69.4712</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>1786.10</t>
+          <t>$1,786.10</t>
         </is>
       </c>
     </row>
@@ -4266,17 +4266,17 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>109300.00</t>
+          <t>$109,300.00</t>
         </is>
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>52.5481</t>
+          <t>$52.5481</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>1062.00</t>
+          <t>$1,062.00</t>
         </is>
       </c>
     </row>
@@ -4351,17 +4351,17 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>61000.00</t>
+          <t>$61,000.00</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>29.3269</t>
+          <t>$29.3269</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>602.96</t>
+          <t>$602.96</t>
         </is>
       </c>
     </row>
@@ -4436,17 +4436,17 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>77650.00</t>
+          <t>$77,650.00</t>
         </is>
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>37.3317</t>
+          <t>$37.3317</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>1383.51</t>
+          <t>$1,383.51</t>
         </is>
       </c>
     </row>
@@ -4521,17 +4521,17 @@
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>108900.00</t>
+          <t>$108,900.00</t>
         </is>
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>52.3558</t>
+          <t>$52.3558</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>1272.77</t>
+          <t>$1,272.77</t>
         </is>
       </c>
     </row>
@@ -4606,17 +4606,17 @@
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>109200.00</t>
+          <t>$109,200.00</t>
         </is>
       </c>
       <c r="P38" t="inlineStr">
         <is>
-          <t>52.5000</t>
+          <t>$52.5000</t>
         </is>
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>830.02</t>
+          <t>$830.02</t>
         </is>
       </c>
     </row>
@@ -4691,17 +4691,17 @@
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>95850.00</t>
+          <t>$95,850.00</t>
         </is>
       </c>
       <c r="P39" t="inlineStr">
         <is>
-          <t>46.0817</t>
+          <t>$46.0817</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>1903.64</t>
+          <t>$1,903.64</t>
         </is>
       </c>
     </row>
@@ -4776,17 +4776,17 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>91200.00</t>
+          <t>$91,200.00</t>
         </is>
       </c>
       <c r="P40" t="inlineStr">
         <is>
-          <t>43.8462</t>
+          <t>$43.8462</t>
         </is>
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>1043.98</t>
+          <t>$1,043.98</t>
         </is>
       </c>
     </row>
@@ -4861,17 +4861,17 @@
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>61900.00</t>
+          <t>$61,900.00</t>
         </is>
       </c>
       <c r="P41" t="inlineStr">
         <is>
-          <t>29.7596</t>
+          <t>$29.7596</t>
         </is>
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>790.41</t>
+          <t>$790.41</t>
         </is>
       </c>
     </row>
@@ -4946,17 +4946,17 @@
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>148200.00</t>
+          <t>$148,200.00</t>
         </is>
       </c>
       <c r="P42" t="inlineStr">
         <is>
-          <t>71.2500</t>
+          <t>$71.2500</t>
         </is>
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>602.78</t>
+          <t>$602.78</t>
         </is>
       </c>
     </row>
@@ -5031,17 +5031,17 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>134000.00</t>
+          <t>$134,000.00</t>
         </is>
       </c>
       <c r="P43" t="inlineStr">
         <is>
-          <t>64.4231</t>
+          <t>$64.4231</t>
         </is>
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>1421.17</t>
+          <t>$1,421.17</t>
         </is>
       </c>
     </row>
@@ -5116,17 +5116,17 @@
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>125600.00</t>
+          <t>$125,600.00</t>
         </is>
       </c>
       <c r="P44" t="inlineStr">
         <is>
-          <t>60.3846</t>
+          <t>$60.3846</t>
         </is>
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>1890.64</t>
+          <t>$1,890.64</t>
         </is>
       </c>
     </row>
@@ -5201,17 +5201,17 @@
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>129750.00</t>
+          <t>$129,750.00</t>
         </is>
       </c>
       <c r="P45" t="inlineStr">
         <is>
-          <t>62.3798</t>
+          <t>$62.3798</t>
         </is>
       </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t>1251.34</t>
+          <t>$1,251.34</t>
         </is>
       </c>
     </row>
@@ -5286,17 +5286,17 @@
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>76850.00</t>
+          <t>$76,850.00</t>
         </is>
       </c>
       <c r="P46" t="inlineStr">
         <is>
-          <t>36.9471</t>
+          <t>$36.9471</t>
         </is>
       </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>159.24</t>
+          <t>$159.24</t>
         </is>
       </c>
     </row>
@@ -5371,17 +5371,17 @@
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>94600.00</t>
+          <t>$94,600.00</t>
         </is>
       </c>
       <c r="P47" t="inlineStr">
         <is>
-          <t>45.4808</t>
+          <t>$45.4808</t>
         </is>
       </c>
       <c r="Q47" t="inlineStr">
         <is>
-          <t>2242.66</t>
+          <t>$2,242.66</t>
         </is>
       </c>
     </row>
@@ -5456,17 +5456,17 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>47840.00</t>
+          <t>$47,840.00</t>
         </is>
       </c>
       <c r="P48" t="inlineStr">
         <is>
-          <t>23.0000</t>
+          <t>$23.0000</t>
         </is>
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>680.80</t>
+          <t>$680.80</t>
         </is>
       </c>
     </row>
@@ -5541,17 +5541,17 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>62450.00</t>
+          <t>$62,450.00</t>
         </is>
       </c>
       <c r="P49" t="inlineStr">
         <is>
-          <t>30.0240</t>
+          <t>$30.0240</t>
         </is>
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>369.60</t>
+          <t>$369.60</t>
         </is>
       </c>
     </row>
@@ -5626,17 +5626,17 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>92000.00</t>
+          <t>$92,000.00</t>
         </is>
       </c>
       <c r="P50" t="inlineStr">
         <is>
-          <t>44.2308</t>
+          <t>$44.2308</t>
         </is>
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>272.02</t>
+          <t>$272.02</t>
         </is>
       </c>
     </row>
@@ -5711,17 +5711,17 @@
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>172500.00</t>
+          <t>$172,500.00</t>
         </is>
       </c>
       <c r="P51" t="inlineStr">
         <is>
-          <t>82.9327</t>
+          <t>$82.9327</t>
         </is>
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>255.43</t>
+          <t>$255.43</t>
         </is>
       </c>
     </row>
@@ -5796,17 +5796,17 @@
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>56300.00</t>
+          <t>$56,300.00</t>
         </is>
       </c>
       <c r="P52" t="inlineStr">
         <is>
-          <t>27.0673</t>
+          <t>$27.0673</t>
         </is>
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>83.37</t>
+          <t>$83.37</t>
         </is>
       </c>
     </row>
@@ -5881,17 +5881,17 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>71900.00</t>
+          <t>$71,900.00</t>
         </is>
       </c>
       <c r="P53" t="inlineStr">
         <is>
-          <t>34.5673</t>
+          <t>$34.5673</t>
         </is>
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>$0.00</t>
         </is>
       </c>
     </row>
@@ -5914,7 +5914,7 @@
       <c r="L54" t="inlineStr"/>
       <c r="M54" t="inlineStr">
         <is>
-          <t>1522.17</t>
+          <t>1,522.17</t>
         </is>
       </c>
       <c r="N54" t="inlineStr"/>
@@ -5922,7 +5922,7 @@
       <c r="P54" t="inlineStr"/>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>92739.54</t>
+          <t>$92,739.54</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
House register: a semicolon or a colon joining clauses is out, a new sentence takes its place
Logged in CLAUDE.md from the show-your-work, whose builder now asserts it with a control.
Every joined clause in the workbook's prose is now its own sentence.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BFcAyctgtHUfeGuTMXxq24
</commit_message>
<xml_diff>
--- a/tasks/HR_Troutly_T2_pto_liability_close/03_show_your_work.xlsx
+++ b/tasks/HR_Troutly_T2_pto_liability_close/03_show_your_work.xlsx
@@ -469,7 +469,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Biweekly accrual at the annual tier over 26, posted on the pay date; carryover capped at 40.0 hours at 06/30/2026; tiers by adjusted service date, the change in the period containing the anniversary; valued at the rate on file over 2,080; ended employees out; wiki pages do not set policy.</t>
+          <t>Biweekly accrual at the annual tier over 26, posted on the pay date. Carryover capped at 40.0 hours at 06/30/2026. Tiers by adjusted service date, the change in the period containing the anniversary. Valued at the rate on file over 2,080. Ended employees out. Wiki pages do not set policy.</t>
         </is>
       </c>
     </row>
@@ -486,7 +486,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Section 7 incorporates the memo; 2.2 part-time accrual pro-rata under 30 hours; 7.6 service bridges on a break under 365 days; 5.4 the $3,000.00 Support Specialist step; 3.2 the signed document over the record; 7.3 totals are the sum of the rounded rows.</t>
+          <t>Section 7 incorporates the memo. 2.2 accrues part-time pro-rata under 30 hours. 7.6 bridges service on a break under 365 days. 5.4 carries the $3,000.00 Support Specialist step. 3.2 puts the signed document over the record. 7.3 totals the rounded rows.</t>
         </is>
       </c>
     </row>
@@ -520,7 +520,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>52 active employees. BambooHR carries 57 active rows: four contractors, three employees whose employment ended 03/20, 05/08 and 06/15/2026, and no row for TRT-0153 and TRT-0155, Never Loaded on the crosswalk.</t>
+          <t>52 active employees. BambooHR carries 57 active rows. Four are contractors, three are employees whose employment ended 03/20, 05/08 and 06/15/2026, and TRT-0153 and TRT-0155 have no row, Never Loaded on the crosswalk.</t>
         </is>
       </c>
     </row>
@@ -537,7 +537,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>51 balances at 06/30/2026; eleven above 40.0 hours, TRT-0005 at 92.50 the highest. The HRIS report, the load file and the July close carry them uncapped.</t>
+          <t>51 balances at 06/30/2026. Eleven are above 40.0 hours, TRT-0005 at 92.50 the highest. The HRIS report, the load file and the July close carry them uncapped.</t>
         </is>
       </c>
     </row>
@@ -554,7 +554,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Pay dates 07/10/2026, 07/24/2026, 08/07/2026 and 08/21/2026, posted by 08/31/2026; 09/04/2026 is the fifth and is not posted.</t>
+          <t>Pay dates 07/10/2026, 07/24/2026, 08/07/2026 and 08/21/2026, posted by 08/31/2026. The fifth pays 09/04/2026 and is not posted.</t>
         </is>
       </c>
     </row>
@@ -571,7 +571,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Nine migrated records read 07/01/2026 in BambooHR and on the roster and carry their true dates in the archive and the letters. TRT-0071 hired 03/08/2021, ended 08/25/2023, rehired 04/22/2024: a break under 365 days, bridged under handbook 7.6.</t>
+          <t>Nine migrated records read 07/01/2026 in BambooHR and on the roster and carry their true dates in the archive and the letters. TRT-0071 was hired 03/08/2021, ended 08/25/2023 and was rehired 04/22/2024, a break under 365 days, bridged under handbook 7.6.</t>
         </is>
       </c>
     </row>
@@ -588,7 +588,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>TRT-0018 reaches five years inside the fourth period: three periods at 120 and one at 160, 20.0000 hours accrued.</t>
+          <t>TRT-0018 reaches five years inside the fourth period. Three periods at 120 and one at 160, 20.0000 hours accrued.</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>TRT-0096 steps $3,000.00 on her 08/17/2026 anniversary: $61,000.00 on file at 08/31/2026.</t>
+          <t>TRT-0096 steps $3,000.00 on her 08/17/2026 anniversary to $61,000.00 on file at 08/31/2026.</t>
         </is>
       </c>
     </row>
@@ -639,7 +639,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>25 hours to 32 hours effective 08/10/2026; pro-rata under 30 hours, so three periods at 25 and one at 32.</t>
+          <t>25 hours to 32 hours effective 08/10/2026. Pro-rata under 30 hours, so three periods at 25 and one at 32.</t>
         </is>
       </c>
     </row>
@@ -656,7 +656,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Okonkwo started 07/22/2026 at $92,000.00, moved from 07/13/2026 by the thread of 07/09/2026; Ibarra 08/03/2026 at $56,300.00. Both accrue at 80 from the period containing the start, as BambooHR credited TRT-0150: 6.15 and 3.08 hours.</t>
+          <t>Okonkwo started 07/22/2026 at $92,000.00, moved from 07/13/2026 by the thread of 07/09/2026. Ibarra started 08/03/2026 at $56,300.00. Both accrue at 80 from the period containing the start, as BambooHR credited TRT-0150, 6.15 and 3.08 hours.</t>
         </is>
       </c>
     </row>
@@ -673,7 +673,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>24 approved requests, 560.00 hours, all in July; TRT-0001 40.00 hours.</t>
+          <t>24 approved requests, 560.00 hours, all in July. TRT-0001 used 40.00 hours.</t>
         </is>
       </c>
     </row>
@@ -690,7 +690,7 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>The requester's method: the HRIS balance, tier and rate per row, three ended employees inside, $90,862.13 booked.</t>
+          <t>The requester's method. The HRIS balance, tier and rate per row, three ended employees inside, $90,862.13 booked.</t>
         </is>
       </c>
     </row>
@@ -1257,7 +1257,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>The determination carries 75 of 92 points; the gate is the total. Every row is read from the Wiki.js pages table or the BambooHR tables.</t>
+          <t>The determination carries 75 of 92 points and the gate is the total. Every row is read from the Wiki.js pages table or the BambooHR tables.</t>
         </is>
       </c>
       <c r="C24" s="2" t="n"/>
@@ -1302,7 +1302,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>52 from the roster and the org chart: BambooHR's 57 active less four contractors less three ended plus the two unloaded hires.</t>
+          <t>52 from the roster and the org chart. BambooHR's 57 active less four contractors less three ended plus the two unloaded hires.</t>
         </is>
       </c>
     </row>
@@ -1314,7 +1314,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>The cutover memo over the 2025 policy and the wiki page; the handbook's bridging, part-time, step and signed-document rules.</t>
+          <t>The cutover memo over the 2025 policy and the wiki page. The handbook's bridging, part-time, step and signed-document rules.</t>
         </is>
       </c>
     </row>
@@ -1326,7 +1326,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>The archive's 06/30/2026 balance capped at 40.00; eleven capped; the two hires at 0.00.</t>
+          <t>The archive's 06/30/2026 balance capped at 40.00. Eleven capped. The two hires at 0.00.</t>
         </is>
       </c>
     </row>
@@ -1338,7 +1338,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>The archive's and the letters' dates over the loaded 07/01/2026; TRT-0071 bridged to 03/08/2021 at 160; five migrated records at 120; TRT-0018 to 160 in the fourth period.</t>
+          <t>The archive's and the letters' dates over the loaded 07/01/2026. TRT-0071 bridged to 03/08/2021 at 160. Five migrated records at 120. TRT-0018 to 160 in the fourth period.</t>
         </is>
       </c>
     </row>
@@ -1350,7 +1350,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Four posted periods at the tier over 26 to four decimals, the period containing a start credited in full; TRT-0141 pro-rata at 25 then 32 hours.</t>
+          <t>Four posted periods at the tier over 26 to four decimals, the period containing a start credited in full. TRT-0141 pro-rata at 25 then 32 hours.</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1374,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>The rate on file over 2,080 to four decimals: TRT-0088 at $118,000.00, TRT-0117 at $148,200.00 and TRT-0096 at $61,000.00 by the signed documents and the step.</t>
+          <t>The rate on file over 2,080 to four decimals. TRT-0088 at $118,000.00, TRT-0117 at $148,200.00 and TRT-0096 at $61,000.00 by the signed documents and the step.</t>
         </is>
       </c>
     </row>
@@ -1386,7 +1386,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Balance to two decimals, liability to the cent, the total the sum of the rounded rows: 1,522.17 hours and $92,739.54, $92,772.88 under posted rounding.</t>
+          <t>Balance to two decimals, liability to the cent, the total the sum of the rounded rows. 1,522.17 hours and $92,739.54, $92,772.88 under posted rounding.</t>
         </is>
       </c>
     </row>
@@ -1398,7 +1398,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>PTO Liability - 08/31/2026: the summary above the table, seven columns, 52 rows keyed by ID, published.</t>
+          <t>PTO Liability - 08/31/2026. The summary above the table, seven columns, 52 rows keyed by ID, published.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
T2: the gate at 10 on the platform's 1 to 10 scale, the plan at 87, every score restated; no Family column
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BFcAyctgtHUfeGuTMXxq24
</commit_message>
<xml_diff>
--- a/tasks/HR_Troutly_T2_pto_liability_close/03_show_your_work.xlsx
+++ b/tasks/HR_Troutly_T2_pto_liability_close/03_show_your_work.xlsx
@@ -722,14 +722,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="110" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -745,15 +744,10 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Family</t>
+          <t>Weight</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Weight</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Gate</t>
         </is>
@@ -768,15 +762,10 @@
           <t>States that a Wiki.js page titled PTO Liability - 08/31/2026 is published.</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>The page and its form</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="n">
+      <c r="C2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -791,15 +780,10 @@
           <t>States, on the PTO liability page, the 52 current employees at 08/31/2026 as the only employee rows.</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>The page and its form</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="n">
+      <c r="C3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -814,15 +798,10 @@
           <t>States, on the PTO liability page, hours to two decimals, hourly rates to four decimals, dollars to the cent and a total equal to the sum of the rows.</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>The page and its form</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="n">
+      <c r="C4" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -837,15 +816,10 @@
           <t>States, on the PTO liability page, a summary with the employee count, the total hours and the total dollar liability.</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>The page and its form</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="n">
+      <c r="C5" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -860,15 +834,10 @@
           <t>States, on the PTO liability page, a total dollar liability of $92,739.54.</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>The determination</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="n">
-        <v>15</v>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="C6" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>Critical value</t>
         </is>
@@ -883,15 +852,10 @@
           <t>States, on the PTO liability page, an opening balance of 40.00 hours for each of the 11 employees whose 06/30/2026 balance exceeded 40.0 hours.</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>The determination</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="n">
+      <c r="C7" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -906,15 +870,10 @@
           <t>States, on the PTO liability page, the 120-hour tier for TRT-0043, TRT-0051, TRT-0058, TRT-0079 and TRT-0083.</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>The determination</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="n">
+      <c r="C8" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -929,15 +888,10 @@
           <t>States, on the PTO liability page, the 160-hour tier for Samuel Burkenham, TRT-0071, with service bridged to 03/08/2021.</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>The determination</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="n">
+      <c r="C9" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -952,15 +906,10 @@
           <t>States, on the PTO liability page, an accrual of 20.0000 hours for Marisela Thornbury, TRT-0018, three periods at the 120-hour tier and one at 160.</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>The determination</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="n">
+      <c r="C10" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -975,15 +924,10 @@
           <t>States, on the PTO liability page, an hourly rate of $56.7308 for Yolanda Featherstone, TRT-0088.</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>The determination</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="n">
+      <c r="C11" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -998,15 +942,10 @@
           <t>States, on the PTO liability page, an hourly rate of $71.2500 for Belaviv Luk, TRT-0117.</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>The determination</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="n">
+      <c r="C12" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1021,15 +960,10 @@
           <t>States, on the PTO liability page, an hourly rate of $29.3269 for Delphine Marchetti, TRT-0096.</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>The determination</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="n">
+      <c r="C13" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1044,15 +978,10 @@
           <t>States, on the PTO liability page, a balance of 29.60 hours for Beatriz Quintanilla, TRT-0141.</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>The determination</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="n">
+      <c r="C14" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1067,15 +996,10 @@
           <t>States, on the PTO liability page, no contractor row, CTR-2001 to CTR-2004.</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>The determination</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="n">
+      <c r="C15" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1090,15 +1014,10 @@
           <t>States, on the PTO liability page, no row for TRT-0037, TRT-0049, TRT-0064 or TRT-0006.</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>The determination</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="n">
+      <c r="C16" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1113,15 +1032,10 @@
           <t>States, on the PTO liability page, Simone Okonkwo, TRT-0153, and Rafael Ibarra, TRT-0155, at the 80-hour tier with accruals since their start dates.</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>The determination</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="n">
+      <c r="C17" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1136,15 +1050,10 @@
           <t>States, on the PTO liability page, a balance of 62.62 hours for Sora Jackson, TRT-0002, four posted periods at the 160-hour tier.</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>The determination</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="n">
+      <c r="C18" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1159,15 +1068,10 @@
           <t>States, on the PTO liability page, a balance of 22.87 hours for Michael Labeson, TRT-0001, with 40.00 hours of approved time off deducted.</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>The determination</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="n">
+      <c r="C19" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1182,15 +1086,10 @@
           <t>States, in BambooHR, the PTO policy the schedule's tier gives for each of the 6 employees whose loaded policy differed.</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>BambooHR brought to the schedule</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="n">
+      <c r="C20" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1205,15 +1104,10 @@
           <t>States, in BambooHR, a PTO balance equal to the schedule's 08/31/2026 balance for every employee on the schedule.</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>BambooHR brought to the schedule</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="n">
+      <c r="C21" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1228,15 +1122,10 @@
           <t>States, in BambooHR, a PTO balance row for TRT-0153 and TRT-0155.</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>BambooHR brought to the schedule</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="n">
+      <c r="C22" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E22" s="2" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -1247,7 +1136,6 @@
       <c r="B23" s="2" t="n"/>
       <c r="C23" s="2" t="n"/>
       <c r="D23" s="2" t="n"/>
-      <c r="E23" s="2" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1257,12 +1145,11 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>The determination carries 75 of 92 points and the gate is the total. Every row is read from the Wiki.js pages table or the BambooHR tables.</t>
+          <t>The determination carries 70 of 87 points and the gate is the total. Every row is read from the Wiki.js pages table or the BambooHR tables.</t>
         </is>
       </c>
       <c r="C24" s="2" t="n"/>
       <c r="D24" s="2" t="n"/>
-      <c r="E24" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
T2: show-your-work notes say what the rows grade, a rule each and never a cell
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BFcAyctgtHUfeGuTMXxq24
</commit_message>
<xml_diff>
--- a/tasks/HR_Troutly_T2_pto_liability_close/03_show_your_work.xlsx
+++ b/tasks/HR_Troutly_T2_pto_liability_close/03_show_your_work.xlsx
@@ -722,7 +722,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1150,6 +1150,62 @@
       </c>
       <c r="C24" s="2" t="n"/>
       <c r="D24" s="2" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Each row grades a rule, and the rule is what a group of cells has in common. A wrong cell is never graded as a wrong cell. It is graded as the rule the run failed to apply, once.</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="n"/>
+      <c r="D25" s="2" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>The gate grades every rule at once through the total, the one number all 364 cells feed. Under the one-cent rule it equals the schedule's only if all 52 liabilities are right.</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="n"/>
+      <c r="D26" s="2" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Rows 6 to 13 each grade one rule on the cells where only that rule moves the value. Rows 2, 14, 15 and 16 grade the population on the set of IDs. Rows 19 to 21 grade BambooHR on its tables.</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="n"/>
+      <c r="D27" s="2" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Drop one rule and one more row fails. The registered paths in 02_task_metadata.md are the proof.</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="n"/>
+      <c r="D28" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
T2: show-your-work notes reworded, a rule graded across its group through a total
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BFcAyctgtHUfeGuTMXxq24
</commit_message>
<xml_diff>
--- a/tasks/HR_Troutly_T2_pto_liability_close/03_show_your_work.xlsx
+++ b/tasks/HR_Troutly_T2_pto_liability_close/03_show_your_work.xlsx
@@ -1159,7 +1159,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Each row grades a rule, and the rule is what a group of cells has in common. A wrong cell is never graded as a wrong cell. It is graded as the rule the run failed to apply, once.</t>
+          <t>Each row grades the correct application of one rule across the group of employees it governs, by reading a total over the group. A total moves if any single entry under it is wrong, so one wrong cell fails the rule once and never twice.</t>
         </is>
       </c>
       <c r="C25" s="2" t="n"/>
@@ -1173,7 +1173,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>The gate grades every rule at once through the total, the one number all 364 cells feed. Under the one-cent rule it equals the schedule's only if all 52 liabilities are right.</t>
+          <t>The gate reads the total of all 52 liabilities, the one number all 364 cells feed. Under the one-cent rule it equals the schedule's only if every entry is right. The witness rows read the cells of the employees their rule alone moves.</t>
         </is>
       </c>
       <c r="C26" s="2" t="n"/>

</xml_diff>

<commit_message>
T2: show-your-work notes, the gate reads the whole group and each witness the employees its rule alone moves
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BFcAyctgtHUfeGuTMXxq24
</commit_message>
<xml_diff>
--- a/tasks/HR_Troutly_T2_pto_liability_close/03_show_your_work.xlsx
+++ b/tasks/HR_Troutly_T2_pto_liability_close/03_show_your_work.xlsx
@@ -1159,7 +1159,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Each row grades the correct application of one rule across the group of employees it governs, by reading a total over the group. A total moves if any single entry under it is wrong, so one wrong cell fails the rule once and never twice.</t>
+          <t>The gate grades every rule across the whole group at once. It reads the total of all 52 liabilities, the one number all 364 cells feed. The reviewer rules allow it one cent of tolerance, and it matches the schedule's within that only if every entry is right.</t>
         </is>
       </c>
       <c r="C25" s="2" t="n"/>
@@ -1173,7 +1173,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>The gate reads the total of all 52 liabilities, the one number all 364 cells feed. The reviewer rules allow it one cent of tolerance, and it matches the schedule's within that only if every entry is right. The witness rows read the cells of the employees their rule alone moves.</t>
+          <t>Each witness row grades one rule on the employees that rule alone moves, so one wrong cell fails a rule once and never twice. Where the rule touches many, the row reads a group, the five capped or the five loaded tiers. Where the world applies it to one person, the bridge, the anniversary, the step and the part-time schedule, the row reads that person. Where it touches everyone, the periods and the usage, one clean witness proves the application.</t>
         </is>
       </c>
       <c r="C26" s="2" t="n"/>
@@ -1187,7 +1187,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Rows 6 to 13 each grade one rule on the cells where only that rule moves the value. Rows 2, 14, 15 and 16 grade the population on the set of IDs. Rows 19 to 21 grade BambooHR on its tables.</t>
+          <t>Rows 2, 14, 15 and 16 grade the population on the set of IDs. Rows 19 to 21 grade BambooHR on its tables.</t>
         </is>
       </c>
       <c r="C27" s="2" t="n"/>

</xml_diff>

<commit_message>
T2: show-your-work notes cut to three, no tolerance and no repo reference
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BFcAyctgtHUfeGuTMXxq24
</commit_message>
<xml_diff>
--- a/tasks/HR_Troutly_T2_pto_liability_close/03_show_your_work.xlsx
+++ b/tasks/HR_Troutly_T2_pto_liability_close/03_show_your_work.xlsx
@@ -722,7 +722,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1145,7 +1145,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>The determination carries 70 of 87 points and the gate is the total. Every row is read from the Wiki.js pages table or the BambooHR tables.</t>
+          <t>The gate grades every rule across the whole group at once. It reads the total of all 52 liabilities, the one number all 364 cells feed, and it matches the schedule's only if every entry is right.</t>
         </is>
       </c>
       <c r="C24" s="2" t="n"/>
@@ -1159,7 +1159,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>The gate grades every rule across the whole group at once. It reads the total of all 52 liabilities, the one number all 364 cells feed. The reviewer rules allow it one cent of tolerance, and it matches the schedule's within that only if every entry is right.</t>
+          <t>Each witness row grades one rule on the employees that rule alone moves, so one wrong cell fails a rule once and never twice. Where the rule touches many, the row reads a group, the five capped or the five loaded tiers. Where the world applies it to one person, the bridge, the anniversary, the step and the part-time schedule, the row reads that person. Where it touches everyone, the periods and the usage, one clean witness proves the application.</t>
         </is>
       </c>
       <c r="C25" s="2" t="n"/>
@@ -1173,39 +1173,11 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Each witness row grades one rule on the employees that rule alone moves, so one wrong cell fails a rule once and never twice. Where the rule touches many, the row reads a group, the five capped or the five loaded tiers. Where the world applies it to one person, the bridge, the anniversary, the step and the part-time schedule, the row reads that person. Where it touches everyone, the periods and the usage, one clean witness proves the application.</t>
+          <t>Rows 2, 14, 15 and 16 grade the population on the set of IDs. Rows 19 to 21 grade BambooHR on its tables.</t>
         </is>
       </c>
       <c r="C26" s="2" t="n"/>
       <c r="D26" s="2" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>Rows 2, 14, 15 and 16 grade the population on the set of IDs. Rows 19 to 21 grade BambooHR on its tables.</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="n"/>
-      <c r="D27" s="2" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-      <c r="B28" s="2" t="inlineStr">
-        <is>
-          <t>Drop one rule and one more row fails. The registered paths in 02_task_metadata.md are the proof.</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="n"/>
-      <c r="D28" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>